<commit_message>
add example for date x
</commit_message>
<xml_diff>
--- a/config/chart_config.xlsx
+++ b/config/chart_config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mpinz-my.sharepoint.com/personal/federico_duranovich_mpi_govt_nz/Documents/Documents/Projects/R projects/autosopi/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="46" documentId="11_B194FE67F1BA918F0CFA9BEF38775098194B2421" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{22520E05-BDE6-4203-B71F-E4E58FAB4A59}"/>
+  <xr:revisionPtr revIDLastSave="169" documentId="11_B194FE67F1BA918F0CFA9BEF38775098194B2421" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4A1AEBDE-E0A8-4159-A136-B334F40731AF}"/>
   <bookViews>
-    <workbookView xWindow="13560" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13560" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -23,12 +23,25 @@
     <sheet name="run_control" sheetId="8" r:id="rId8"/>
     <sheet name="palettes" sheetId="9" r:id="rId9"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="610" uniqueCount="239">
   <si>
     <t>Purpose</t>
   </si>
@@ -177,9 +190,6 @@
     <t>Macro</t>
   </si>
   <si>
-    <t>2018</t>
-  </si>
-  <si>
     <t>macro_palette</t>
   </si>
   <si>
@@ -189,9 +199,6 @@
     <t>Seafood</t>
   </si>
   <si>
-    <t>2020</t>
-  </si>
-  <si>
     <t>seafood_palette</t>
   </si>
   <si>
@@ -646,13 +653,118 @@
   </si>
   <si>
     <t>#56CCF2</t>
+  </si>
+  <si>
+    <t>Horticulture</t>
+  </si>
+  <si>
+    <t>horticulture_pallete</t>
+  </si>
+  <si>
+    <t>kiwifruit_comb</t>
+  </si>
+  <si>
+    <t>generic_ts_plot</t>
+  </si>
+  <si>
+    <t>kiwifruit_fig_1</t>
+  </si>
+  <si>
+    <t>kiwifruit_fig_1.svg</t>
+  </si>
+  <si>
+    <t>Kwiwifuit</t>
+  </si>
+  <si>
+    <t>data/raw/manual_data.xlsx</t>
+  </si>
+  <si>
+    <t>financial_year</t>
+  </si>
+  <si>
+    <t>revenue</t>
+  </si>
+  <si>
+    <t>Export revenue (NZ$ million)</t>
+  </si>
+  <si>
+    <t>volume_mn_trays</t>
+  </si>
+  <si>
+    <t>col_position</t>
+  </si>
+  <si>
+    <t>dodge</t>
+  </si>
+  <si>
+    <t>category</t>
+  </si>
+  <si>
+    <t>forecast</t>
+  </si>
+  <si>
+    <t>forecast_start</t>
+  </si>
+  <si>
+    <t>forecast_end</t>
+  </si>
+  <si>
+    <t>#c49a00</t>
+  </si>
+  <si>
+    <t>gold</t>
+  </si>
+  <si>
+    <t>green</t>
+  </si>
+  <si>
+    <t>#1e8449</t>
+  </si>
+  <si>
+    <t>other</t>
+  </si>
+  <si>
+    <t>#4d4d4d</t>
+  </si>
+  <si>
+    <t>kiwifruit_comb2</t>
+  </si>
+  <si>
+    <t>kiwifruit_fig_2.svg</t>
+  </si>
+  <si>
+    <t>stacked</t>
+  </si>
+  <si>
+    <t>line_label</t>
+  </si>
+  <si>
+    <t>Volume</t>
+  </si>
+  <si>
+    <t>col_label</t>
+  </si>
+  <si>
+    <t>Revenue</t>
+  </si>
+  <si>
+    <t>seafood_1</t>
+  </si>
+  <si>
+    <t>volume</t>
+  </si>
+  <si>
+    <t>seafood_fig_1</t>
+  </si>
+  <si>
+    <t>seafood_fig_1.svg</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -661,6 +773,10 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Carlito"/>
     </font>
   </fonts>
@@ -677,7 +793,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -700,16 +816,28 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9E2F3"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9E2F3"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -943,7 +1071,7 @@
     <col min="4" max="4" width="31.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="28">
+    <row r="1" spans="1:4">
       <c r="A1" s="2" t="s">
         <v>10</v>
       </c>
@@ -1094,10 +1222,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="7.75" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.08203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="6.58203125" customWidth="1"/>
     <col min="3" max="3" width="9.58203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9" bestFit="1" customWidth="1"/>
@@ -1106,7 +1234,7 @@
     <col min="7" max="7" width="28.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="28">
+    <row r="1" spans="1:7">
       <c r="A1" s="2" t="s">
         <v>45</v>
       </c>
@@ -1136,89 +1264,109 @@
       <c r="B2" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="1">
+        <v>2026</v>
+      </c>
+      <c r="D2" s="1">
+        <v>2030</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>50</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>48</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="1">
+        <v>2026</v>
+      </c>
+      <c r="D3" s="1">
+        <v>2030</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="G3" s="1" t="s">
         <v>53</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>33</v>
+      <c r="C4" s="1">
+        <v>2026</v>
+      </c>
+      <c r="D4" s="1">
+        <v>2030</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F4" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G4" s="1" t="s">
         <v>56</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C5" s="1">
+        <v>2026</v>
+      </c>
+      <c r="D5" s="1">
+        <v>2030</v>
+      </c>
+      <c r="E5" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="F5" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="G5" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>62</v>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="B6" t="b">
+        <v>1</v>
+      </c>
+      <c r="C6" s="1">
+        <v>2026</v>
+      </c>
+      <c r="D6" s="1">
+        <v>2030</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>204</v>
       </c>
     </row>
   </sheetData>
@@ -1232,7 +1380,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="22.25" bestFit="1" customWidth="1"/>
@@ -1247,9 +1395,9 @@
     <col min="10" max="10" width="29.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="28">
+    <row r="1" spans="1:10">
       <c r="A1" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>45</v>
@@ -1258,22 +1406,22 @@
         <v>46</v>
       </c>
       <c r="D1" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>67</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>69</v>
       </c>
       <c r="J1" s="2" t="s">
         <v>13</v>
@@ -1281,7 +1429,7 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>48</v>
@@ -1290,30 +1438,30 @@
         <v>42</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>75</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="3" spans="1:10">
       <c r="A3" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>48</v>
@@ -1322,92 +1470,168 @@
         <v>42</v>
       </c>
       <c r="D3" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="I3" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="J3" s="1" t="s">
         <v>83</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" s="1" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>42</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E4" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="G4" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="H4" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="I4" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J4" s="1" t="s">
         <v>89</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="1" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>42</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E5" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G5" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="H5" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="I5" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J5" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="H5" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>97</v>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="C6" t="b">
+        <v>1</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="I6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10">
+      <c r="A7" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="C7" t="b">
+        <v>1</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="I7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10">
+      <c r="A8" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C8" t="b">
+        <v>1</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="I8">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;"Aptos"&amp;12&amp;K000000 UNCLASSIFIED&amp;1#_x000D_</oddHeader>
@@ -1418,27 +1642,28 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E66"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="3" width="18" customWidth="1"/>
+    <col min="1" max="1" width="22.25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="24.08203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8.58203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21.9140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="28">
+    <row r="1" spans="1:5">
       <c r="A1" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>114</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>116</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>13</v>
@@ -1446,180 +1671,180 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>127</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" s="1" t="s">
         <v>130</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>133</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>30</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>30</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>30</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>26</v>
@@ -1628,202 +1853,202 @@
         <v>30</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B13" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="D13" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="C13" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>119</v>
-      </c>
       <c r="E13" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>30</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>16</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="1" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B17" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D17" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="E17" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="1" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="1" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="1" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="1" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B21" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E21" s="1" t="s">
         <v>127</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="1" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>30</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="1" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>30</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="24" spans="1:5">
       <c r="A24" s="1" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>26</v>
@@ -1832,134 +2057,134 @@
         <v>30</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" s="1" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D25" s="1" t="s">
         <v>30</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" s="1" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B26" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D26" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="E26" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="1" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="1" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="1" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B29" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E29" s="1" t="s">
         <v>127</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="1" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="D30" s="1" t="s">
         <v>16</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="1" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D31" s="1" t="s">
         <v>30</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="32" spans="1:5">
       <c r="A32" s="1" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>26</v>
@@ -1968,10 +2193,487 @@
         <v>30</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>154</v>
+        <v>152</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4">
+      <c r="A33" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C33" t="s">
+        <v>212</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4">
+      <c r="A34" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C34" t="s">
+        <v>213</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4">
+      <c r="A35" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4">
+      <c r="A36" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="B36" t="s">
+        <v>233</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4">
+      <c r="A37" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C37" t="s">
+        <v>215</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4">
+      <c r="A38" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C38" t="s">
+        <v>132</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4">
+      <c r="A39" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="B39" t="s">
+        <v>231</v>
+      </c>
+      <c r="C39" t="s">
+        <v>232</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4">
+      <c r="A40" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="B40" t="s">
+        <v>216</v>
+      </c>
+      <c r="C40" t="s">
+        <v>217</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4">
+      <c r="A41" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="B41" t="s">
+        <v>123</v>
+      </c>
+      <c r="C41" t="s">
+        <v>218</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4">
+      <c r="A42" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="B42" t="s">
+        <v>219</v>
+      </c>
+      <c r="C42" t="b">
+        <v>1</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4">
+      <c r="A43" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="B43" t="s">
+        <v>220</v>
+      </c>
+      <c r="C43">
+        <v>2026</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4">
+      <c r="A44" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="B44" t="s">
+        <v>221</v>
+      </c>
+      <c r="C44">
+        <v>2030</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4">
+      <c r="A45" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C45" t="s">
+        <v>212</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4">
+      <c r="A46" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C46" t="s">
+        <v>213</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4">
+      <c r="A47" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4">
+      <c r="A48" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C48" t="s">
+        <v>215</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4">
+      <c r="A49" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C49" t="s">
+        <v>132</v>
+      </c>
+      <c r="D49" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4">
+      <c r="A50" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="B50" t="s">
+        <v>216</v>
+      </c>
+      <c r="C50" t="s">
+        <v>230</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4">
+      <c r="A51" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="B51" t="s">
+        <v>123</v>
+      </c>
+      <c r="C51" t="s">
+        <v>218</v>
+      </c>
+      <c r="D51" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4">
+      <c r="A52" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="B52" t="s">
+        <v>219</v>
+      </c>
+      <c r="C52" t="b">
+        <v>1</v>
+      </c>
+      <c r="D52" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4">
+      <c r="A53" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="B53" t="s">
+        <v>220</v>
+      </c>
+      <c r="C53">
+        <v>2026</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4">
+      <c r="A54" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="B54" t="s">
+        <v>221</v>
+      </c>
+      <c r="C54">
+        <v>2030</v>
+      </c>
+      <c r="D54" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4">
+      <c r="A55" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C55" t="s">
+        <v>116</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4">
+      <c r="A56" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C56" t="s">
+        <v>213</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4">
+      <c r="A57" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4">
+      <c r="A58" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="B58" t="s">
+        <v>233</v>
+      </c>
+      <c r="C58" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4">
+      <c r="A59" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C59" t="s">
+        <v>236</v>
+      </c>
+      <c r="D59" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4">
+      <c r="A60" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C60" t="s">
+        <v>132</v>
+      </c>
+      <c r="D60" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4">
+      <c r="A61" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="B61" t="s">
+        <v>231</v>
+      </c>
+      <c r="C61" t="s">
+        <v>232</v>
+      </c>
+      <c r="D61" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4">
+      <c r="A62" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="B62" t="s">
+        <v>216</v>
+      </c>
+      <c r="C62" t="s">
+        <v>217</v>
+      </c>
+      <c r="D62" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4">
+      <c r="A63" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="B63" t="s">
+        <v>123</v>
+      </c>
+      <c r="C63" t="s">
+        <v>123</v>
+      </c>
+      <c r="D63" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4">
+      <c r="A64" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="B64" t="s">
+        <v>219</v>
+      </c>
+      <c r="C64" t="b">
+        <v>1</v>
+      </c>
+      <c r="D64" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4">
+      <c r="A65" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="B65" t="s">
+        <v>220</v>
+      </c>
+      <c r="C65">
+        <v>2026</v>
+      </c>
+      <c r="D65" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4">
+      <c r="A66" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="B66" t="s">
+        <v>221</v>
+      </c>
+      <c r="C66">
+        <v>2030</v>
+      </c>
+      <c r="D66" s="3" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;"Aptos"&amp;12&amp;K000000 UNCLASSIFIED&amp;1#_x000D_</oddHeader>
@@ -1982,7 +2684,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="20.6640625" customWidth="1"/>
@@ -1997,25 +2699,25 @@
   <sheetData>
     <row r="1" spans="1:8" ht="28">
       <c r="A1" s="2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>101</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>103</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>13</v>
@@ -2023,89 +2725,144 @@
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
       <c r="F3" s="1" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="1" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>108</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>110</v>
       </c>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" s="1" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
       <c r="G5" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>113</v>
+        <v>111</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>237</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;"Aptos"&amp;12&amp;K000000 UNCLASSIFIED&amp;1#_x000D_</oddHeader>
@@ -2119,25 +2876,25 @@
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="20.6640625" customWidth="1"/>
-    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="1" max="1" width="23.25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="44.6640625" customWidth="1"/>
     <col min="4" max="4" width="13.25" customWidth="1"/>
     <col min="5" max="5" width="19.4140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="28">
+    <row r="1" spans="1:5">
       <c r="A1" s="2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>114</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>116</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>13</v>
@@ -2145,7 +2902,7 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>45</v>
@@ -2157,46 +2914,46 @@
         <v>16</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>157</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>30</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>45</v>
@@ -2208,41 +2965,41 @@
         <v>16</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>30</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
   </sheetData>
@@ -2265,7 +3022,7 @@
     <col min="4" max="4" width="49.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="28">
+    <row r="1" spans="1:4">
       <c r="A1" s="2" t="s">
         <v>10</v>
       </c>
@@ -2281,7 +3038,7 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="1" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>42</v>
@@ -2290,50 +3047,50 @@
         <v>43</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="1" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="1" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B4" s="1"/>
       <c r="C4" s="1" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="1" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>43</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="1" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>42</v>
@@ -2342,7 +3099,7 @@
         <v>43</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
   </sheetData>
@@ -2356,10 +3113,10 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="12.6640625" customWidth="1"/>
+    <col min="1" max="1" width="16.25" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.1640625" customWidth="1"/>
     <col min="3" max="3" width="7.4140625" customWidth="1"/>
     <col min="4" max="4" width="12.6640625" customWidth="1"/>
@@ -2370,10 +3127,10 @@
         <v>35</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>13</v>
@@ -2384,13 +3141,13 @@
         <v>36</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>178</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -2398,13 +3155,13 @@
         <v>36</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -2412,24 +3169,24 @@
         <v>36</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>48</v>
@@ -2437,13 +3194,13 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>48</v>
@@ -2451,13 +3208,13 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>48</v>
@@ -2465,128 +3222,161 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="C16" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="D16" s="1" t="s">
-        <v>59</v>
+      <c r="B17" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="C17" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="C18" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="C19" t="s">
+        <v>227</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Meat and Wool config test plot
</commit_message>
<xml_diff>
--- a/config/chart_config.xlsx
+++ b/config/chart_config.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Ra87d2b08d9774b53"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="release_settings" sheetId="2" r:id="R1d7a330304d743c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings_sector" sheetId="3" r:id="R97dd0dc5b1d24322"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="plots" sheetId="4" r:id="Rfdae251284364d53"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="plot_args" sheetId="5" r:id="Rc2a9bd1935444248"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="data_sources" sheetId="6" r:id="R3fca647843ec4581"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="data_args" sheetId="7" r:id="R82e750bf211f46f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="run_control" sheetId="8" r:id="Reb93d27642e64ee6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="palettes" sheetId="9" r:id="R240b3e9f5c1f47cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R70f8c47360684ea7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="release_settings" sheetId="2" r:id="Rec69d9b453174cfd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings_sector" sheetId="3" r:id="R10c5dcac39944ddf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="plots" sheetId="4" r:id="R4ab45f9b4cc94f02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="plot_args" sheetId="5" r:id="Red25ad93854f44f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="data_sources" sheetId="6" r:id="Re560c8c693e94808"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="data_args" sheetId="7" r:id="Rccf868791976486b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="run_control" sheetId="8" r:id="R11cb6ffc55d94d63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="palettes" sheetId="9" r:id="R8e9d69402edb4fd5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -308,7 +308,7 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="22.5" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="90.12999725341797" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="94.12999725341797" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -352,26 +352,26 @@
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" t="str">
+      <x:c r="A6" s="1" t="str">
         <x:v>Forecast years</x:v>
       </x:c>
-      <x:c r="B6" t="str">
+      <x:c r="B6" s="1" t="str">
         <x:v>Most plots inherit forecast_start_year and forecast_end_year from release_settings. Override in plot_args only for exceptions.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" t="str">
+      <x:c r="A7" s="1" t="str">
         <x:v>Data sources</x:v>
       </x:c>
-      <x:c r="B7" t="str">
+      <x:c r="B7" s="1" t="str">
         <x:v>source_type excel reads data/raw workbooks; source_type function calls an R function listed in data_function.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" t="str">
+      <x:c r="A8" s="1" t="str">
         <x:v>Column names</x:v>
       </x:c>
-      <x:c r="B8" t="str">
+      <x:c r="B8" s="1" t="str">
         <x:v>Use plain string names in x, y, y_line, y_col, and group arguments.</x:v>
       </x:c>
     </x:row>
@@ -595,11 +595,11 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="9.630000114440918" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="5" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="15.380000114440918" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="13.630000114440918" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="24.1299991607666" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="34.880001068115234" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -701,6 +701,21 @@
         <x:v>Horticulture</x:v>
       </x:c>
       <x:c r="E6" s="1"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="1" t="str">
+        <x:v>Meat and Wool</x:v>
+      </x:c>
+      <x:c r="B7" s="6" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C7" s="1"/>
+      <x:c r="D7" s="1" t="str">
+        <x:v>Meat and Wool</x:v>
+      </x:c>
+      <x:c r="E7" s="1" t="str">
+        <x:v>Function-backed fake Meat and Wool test plot</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -712,15 +727,15 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="9.630000114440918" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="5" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="12.880000114440918" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="20.6299991607666" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="22.75" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="27.5" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="31.25" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="44.630001068115234" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="8.5" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="25.8799991607666" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="36" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -990,6 +1005,38 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="J9" s="1"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="1" t="str">
+        <x:v>meat_wool_fake_ts</x:v>
+      </x:c>
+      <x:c r="B10" s="1" t="str">
+        <x:v>Meat and Wool</x:v>
+      </x:c>
+      <x:c r="C10" s="6" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D10" s="1" t="str">
+        <x:v>generic_ts_plot</x:v>
+      </x:c>
+      <x:c r="E10" s="1" t="str">
+        <x:v>meat_wool_fake</x:v>
+      </x:c>
+      <x:c r="F10" s="1" t="str">
+        <x:v>meat_wool_fig_1.svg</x:v>
+      </x:c>
+      <x:c r="G10" s="1" t="str">
+        <x:v>Meat and Wool fake revenue and volume</x:v>
+      </x:c>
+      <x:c r="H10" s="1" t="str">
+        <x:v>Generated from metadata forecast groups</x:v>
+      </x:c>
+      <x:c r="I10" s="1" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J10" s="1" t="str">
+        <x:v>Function-backed test using metadata categories</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2121,6 +2168,231 @@
       </x:c>
       <x:c r="E70" s="1"/>
     </x:row>
+    <x:row r="71">
+      <x:c r="A71" s="1" t="str">
+        <x:v>meat_wool_fake_ts</x:v>
+      </x:c>
+      <x:c r="B71" s="1" t="str">
+        <x:v>x</x:v>
+      </x:c>
+      <x:c r="C71" s="1" t="str">
+        <x:v>year</x:v>
+      </x:c>
+      <x:c r="D71" s="1" t="str">
+        <x:v>character</x:v>
+      </x:c>
+      <x:c r="E71" s="1"/>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" s="1" t="str">
+        <x:v>meat_wool_fake_ts</x:v>
+      </x:c>
+      <x:c r="B72" s="1" t="str">
+        <x:v>y_col</x:v>
+      </x:c>
+      <x:c r="C72" s="1" t="str">
+        <x:v>revenue</x:v>
+      </x:c>
+      <x:c r="D72" s="1" t="str">
+        <x:v>character</x:v>
+      </x:c>
+      <x:c r="E72" s="1"/>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" s="1" t="str">
+        <x:v>meat_wool_fake_ts</x:v>
+      </x:c>
+      <x:c r="B73" s="1" t="str">
+        <x:v>y_col_label</x:v>
+      </x:c>
+      <x:c r="C73" s="1" t="str">
+        <x:v>Export revenue (NZ$ million)</x:v>
+      </x:c>
+      <x:c r="D73" s="1" t="str">
+        <x:v>character</x:v>
+      </x:c>
+      <x:c r="E73" s="1"/>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" s="1" t="str">
+        <x:v>meat_wool_fake_ts</x:v>
+      </x:c>
+      <x:c r="B74" s="1" t="str">
+        <x:v>col_label</x:v>
+      </x:c>
+      <x:c r="C74" s="1" t="str">
+        <x:v>Revenue</x:v>
+      </x:c>
+      <x:c r="D74" s="1" t="str">
+        <x:v>character</x:v>
+      </x:c>
+      <x:c r="E74" s="1"/>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" s="1" t="str">
+        <x:v>meat_wool_fake_ts</x:v>
+      </x:c>
+      <x:c r="B75" s="1" t="str">
+        <x:v>y_line</x:v>
+      </x:c>
+      <x:c r="C75" s="1" t="str">
+        <x:v>volume</x:v>
+      </x:c>
+      <x:c r="D75" s="1" t="str">
+        <x:v>character</x:v>
+      </x:c>
+      <x:c r="E75" s="1"/>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" s="1" t="str">
+        <x:v>meat_wool_fake_ts</x:v>
+      </x:c>
+      <x:c r="B76" s="1" t="str">
+        <x:v>y_line_label</x:v>
+      </x:c>
+      <x:c r="C76" s="1" t="str">
+        <x:v>Export volume (tonnes)</x:v>
+      </x:c>
+      <x:c r="D76" s="1" t="str">
+        <x:v>character</x:v>
+      </x:c>
+      <x:c r="E76" s="1"/>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" s="1" t="str">
+        <x:v>meat_wool_fake_ts</x:v>
+      </x:c>
+      <x:c r="B77" s="1" t="str">
+        <x:v>line_label</x:v>
+      </x:c>
+      <x:c r="C77" s="1" t="str">
+        <x:v>Volume</x:v>
+      </x:c>
+      <x:c r="D77" s="1" t="str">
+        <x:v>character</x:v>
+      </x:c>
+      <x:c r="E77" s="1"/>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78" s="1" t="str">
+        <x:v>meat_wool_fake_ts</x:v>
+      </x:c>
+      <x:c r="B78" s="1" t="str">
+        <x:v>x_freq</x:v>
+      </x:c>
+      <x:c r="C78" s="1" t="str">
+        <x:v>yearly</x:v>
+      </x:c>
+      <x:c r="D78" s="1" t="str">
+        <x:v>character</x:v>
+      </x:c>
+      <x:c r="E78" s="1"/>
+    </x:row>
+    <x:row r="79">
+      <x:c r="A79" s="1" t="str">
+        <x:v>meat_wool_fake_ts</x:v>
+      </x:c>
+      <x:c r="B79" s="1" t="str">
+        <x:v>col_position</x:v>
+      </x:c>
+      <x:c r="C79" s="1" t="str">
+        <x:v>stacked</x:v>
+      </x:c>
+      <x:c r="D79" s="1" t="str">
+        <x:v>character</x:v>
+      </x:c>
+      <x:c r="E79" s="1"/>
+    </x:row>
+    <x:row r="80">
+      <x:c r="A80" s="1" t="str">
+        <x:v>meat_wool_fake_ts</x:v>
+      </x:c>
+      <x:c r="B80" s="1" t="str">
+        <x:v>group</x:v>
+      </x:c>
+      <x:c r="C80" s="1" t="str">
+        <x:v>group</x:v>
+      </x:c>
+      <x:c r="D80" s="1" t="str">
+        <x:v>character</x:v>
+      </x:c>
+      <x:c r="E80" s="1"/>
+    </x:row>
+    <x:row r="81">
+      <x:c r="A81" s="1" t="str">
+        <x:v>meat_wool_fake_ts</x:v>
+      </x:c>
+      <x:c r="B81" s="1" t="str">
+        <x:v>forecast</x:v>
+      </x:c>
+      <x:c r="C81" s="6" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D81" s="1" t="str">
+        <x:v>logical</x:v>
+      </x:c>
+      <x:c r="E81" s="1"/>
+    </x:row>
+    <x:row r="82">
+      <x:c r="A82" s="1" t="str">
+        <x:v>meat_wool_fake_ts</x:v>
+      </x:c>
+      <x:c r="B82" s="1" t="str">
+        <x:v>primary_min_breaks</x:v>
+      </x:c>
+      <x:c r="C82" s="1" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D82" s="1" t="str">
+        <x:v>integer</x:v>
+      </x:c>
+      <x:c r="E82" s="1"/>
+    </x:row>
+    <x:row r="83">
+      <x:c r="A83" s="1" t="str">
+        <x:v>meat_wool_fake_ts</x:v>
+      </x:c>
+      <x:c r="B83" s="1" t="str">
+        <x:v>primary_max_breaks</x:v>
+      </x:c>
+      <x:c r="C83" s="1" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D83" s="1" t="str">
+        <x:v>integer</x:v>
+      </x:c>
+      <x:c r="E83" s="1"/>
+    </x:row>
+    <x:row r="84">
+      <x:c r="A84" s="1" t="str">
+        <x:v>meat_wool_fake_ts</x:v>
+      </x:c>
+      <x:c r="B84" s="1" t="str">
+        <x:v>secondary_min_breaks</x:v>
+      </x:c>
+      <x:c r="C84" s="1" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D84" s="1" t="str">
+        <x:v>integer</x:v>
+      </x:c>
+      <x:c r="E84" s="1"/>
+    </x:row>
+    <x:row r="85">
+      <x:c r="A85" s="1" t="str">
+        <x:v>meat_wool_fake_ts</x:v>
+      </x:c>
+      <x:c r="B85" s="1" t="str">
+        <x:v>secondary_max_breaks</x:v>
+      </x:c>
+      <x:c r="C85" s="1" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D85" s="1" t="str">
+        <x:v>integer</x:v>
+      </x:c>
+      <x:c r="E85" s="1"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2135,9 +2407,9 @@
     <x:col min="3" max="3" width="26.3799991607666" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="15.130000114440918" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="4.75" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="22.1299991607666" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="26" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="4.880000114440918" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="23" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="51" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -2329,6 +2601,26 @@
       <x:c r="F9" s="1"/>
       <x:c r="G9" s="1"/>
       <x:c r="H9" s="1"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="1" t="str">
+        <x:v>meat_wool_fake</x:v>
+      </x:c>
+      <x:c r="B10" s="1" t="str">
+        <x:v>function</x:v>
+      </x:c>
+      <x:c r="C10" s="1"/>
+      <x:c r="D10" s="1"/>
+      <x:c r="E10" s="1"/>
+      <x:c r="F10" s="1" t="str">
+        <x:v>prep_fake_meat_wool_timeseries</x:v>
+      </x:c>
+      <x:c r="G10" s="6" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H10" s="1" t="str">
+        <x:v>Generated fake Meat and Wool data from metadata forecast groups</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2465,6 +2757,40 @@
         <x:v>Reproducible fake data</x:v>
       </x:c>
     </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="1" t="str">
+        <x:v>meat_wool_fake</x:v>
+      </x:c>
+      <x:c r="B8" s="1" t="str">
+        <x:v>sector</x:v>
+      </x:c>
+      <x:c r="C8" s="1" t="str">
+        <x:v>Meat and Wool</x:v>
+      </x:c>
+      <x:c r="D8" s="1" t="str">
+        <x:v>character</x:v>
+      </x:c>
+      <x:c r="E8" s="1" t="str">
+        <x:v>Metadata sector key</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="1" t="str">
+        <x:v>meat_wool_fake</x:v>
+      </x:c>
+      <x:c r="B9" s="1" t="str">
+        <x:v>seed</x:v>
+      </x:c>
+      <x:c r="C9" s="1" t="n">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="D9" s="1" t="str">
+        <x:v>integer</x:v>
+      </x:c>
+      <x:c r="E9" s="1" t="str">
+        <x:v>Reproducible fake data</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Fix metadata palette resolution
</commit_message>
<xml_diff>
--- a/config/chart_config.xlsx
+++ b/config/chart_config.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R70f8c47360684ea7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="release_settings" sheetId="2" r:id="Rec69d9b453174cfd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings_sector" sheetId="3" r:id="R10c5dcac39944ddf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="plots" sheetId="4" r:id="R4ab45f9b4cc94f02"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="plot_args" sheetId="5" r:id="Red25ad93854f44f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="data_sources" sheetId="6" r:id="Re560c8c693e94808"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="data_args" sheetId="7" r:id="Rccf868791976486b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="run_control" sheetId="8" r:id="R11cb6ffc55d94d63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="palettes" sheetId="9" r:id="R8e9d69402edb4fd5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rbdfd6798a22e460b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="release_settings" sheetId="2" r:id="R40f10319d4b04b4c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings_sector" sheetId="3" r:id="Ra0c90753393e4aa3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="plots" sheetId="4" r:id="R5ac18cbf4f0540a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="plot_args" sheetId="5" r:id="Rfdf8c2f1d0264478"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="data_sources" sheetId="6" r:id="R0e6526bc94ca4f61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="data_args" sheetId="7" r:id="Raa7f7b73b85d41cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="run_control" sheetId="8" r:id="R20e4d2dbff0d4f4c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="palettes" sheetId="9" r:id="R6ee5e0a4c8334f3e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2393,6 +2393,40 @@
       </x:c>
       <x:c r="E85" s="1"/>
     </x:row>
+    <x:row r="86">
+      <x:c r="A86" t="str">
+        <x:v>seafood_1</x:v>
+      </x:c>
+      <x:c r="B86" t="str">
+        <x:v>use_metadata_palette</x:v>
+      </x:c>
+      <x:c r="C86" s="5" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D86" t="str">
+        <x:v>logical</x:v>
+      </x:c>
+      <x:c r="E86" t="str">
+        <x:v>Use metadata forecast-group colours instead of inherited sector palette</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87">
+      <x:c r="A87" t="str">
+        <x:v>seafood_2</x:v>
+      </x:c>
+      <x:c r="B87" t="str">
+        <x:v>use_metadata_palette</x:v>
+      </x:c>
+      <x:c r="C87" s="5" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D87" t="str">
+        <x:v>logical</x:v>
+      </x:c>
+      <x:c r="E87" t="str">
+        <x:v>Use metadata forecast-group colours instead of inherited sector palette</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>